<commit_message>
Chapter 2: matched-window house price data, discrete/continuous section, Excel demo workbooks
</commit_message>
<xml_diff>
--- a/data/ch02-frequency-BROKEN.xlsx
+++ b/data/ch02-frequency-BROKEN.xlsx
@@ -613,7 +613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:N51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -628,6 +628,8 @@
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -653,40 +655,50 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>gHPI5</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>nDOWN</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>UR</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>POPN</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>POPO</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>gPOP</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>HPI_date</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>HPIO_date</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>UR_date</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>POP_date</t>
         </is>
@@ -708,33 +720,39 @@
         <v>88.59999999999999</v>
       </c>
       <c r="E2" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="F2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G2" t="n">
         <v>3.2</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H2" t="n">
         <v>5193.088</v>
       </c>
-      <c r="G2" t="n">
+      <c r="I2" t="n">
         <v>4854.803</v>
       </c>
-      <c r="H2" t="n">
+      <c r="J2" t="n">
         <v>7</v>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -756,33 +774,39 @@
         <v>59.3</v>
       </c>
       <c r="E3" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>7</v>
+      </c>
+      <c r="G3" t="n">
         <v>4.4</v>
       </c>
-      <c r="F3" t="n">
+      <c r="H3" t="n">
         <v>737.27</v>
       </c>
-      <c r="G3" t="n">
+      <c r="I3" t="n">
         <v>738.4299999999999</v>
       </c>
-      <c r="H3" t="n">
+      <c r="J3" t="n">
         <v>-0.2</v>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -804,33 +828,39 @@
         <v>121.5</v>
       </c>
       <c r="E4" t="n">
+        <v>47.7</v>
+      </c>
+      <c r="F4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G4" t="n">
         <v>4.9</v>
       </c>
-      <c r="F4" t="n">
+      <c r="H4" t="n">
         <v>7623.818</v>
       </c>
-      <c r="G4" t="n">
+      <c r="I4" t="n">
         <v>6832.81</v>
       </c>
-      <c r="H4" t="n">
+      <c r="J4" t="n">
         <v>11.6</v>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -852,33 +882,39 @@
         <v>88.3</v>
       </c>
       <c r="E5" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
         <v>4.1</v>
       </c>
-      <c r="F5" t="n">
+      <c r="H5" t="n">
         <v>3114.791</v>
       </c>
-      <c r="G5" t="n">
+      <c r="I5" t="n">
         <v>2979.732</v>
       </c>
-      <c r="H5" t="n">
+      <c r="J5" t="n">
         <v>4.5</v>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -900,33 +936,39 @@
         <v>79.59999999999999</v>
       </c>
       <c r="E6" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="F6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" t="n">
         <v>5.2</v>
       </c>
-      <c r="F6" t="n">
+      <c r="H6" t="n">
         <v>39355.309</v>
       </c>
-      <c r="G6" t="n">
+      <c r="I6" t="n">
         <v>38904.296</v>
       </c>
-      <c r="H6" t="n">
+      <c r="J6" t="n">
         <v>1.2</v>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -948,33 +990,39 @@
         <v>92.09999999999999</v>
       </c>
       <c r="E7" t="n">
+        <v>34.3</v>
+      </c>
+      <c r="F7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" t="n">
         <v>3.9</v>
       </c>
-      <c r="F7" t="n">
+      <c r="H7" t="n">
         <v>6012.561</v>
       </c>
-      <c r="G7" t="n">
+      <c r="I7" t="n">
         <v>5454.328</v>
       </c>
-      <c r="H7" t="n">
+      <c r="J7" t="n">
         <v>10.2</v>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -996,33 +1044,39 @@
         <v>87.5</v>
       </c>
       <c r="E8" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="F8" t="n">
+        <v>5</v>
+      </c>
+      <c r="G8" t="n">
         <v>5.2</v>
       </c>
-      <c r="F8" t="n">
+      <c r="H8" t="n">
         <v>3688.496</v>
       </c>
-      <c r="G8" t="n">
+      <c r="I8" t="n">
         <v>3588.561</v>
       </c>
-      <c r="H8" t="n">
+      <c r="J8" t="n">
         <v>2.8</v>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -1044,33 +1098,39 @@
         <v>81.5</v>
       </c>
       <c r="E9" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" t="n">
         <v>4.9</v>
       </c>
-      <c r="F9" t="n">
+      <c r="H9" t="n">
         <v>1059.952</v>
       </c>
-      <c r="G9" t="n">
+      <c r="I9" t="n">
         <v>942.0650000000001</v>
       </c>
-      <c r="H9" t="n">
+      <c r="J9" t="n">
         <v>12.5</v>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -1092,33 +1152,39 @@
         <v>126.1</v>
       </c>
       <c r="E10" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4</v>
+      </c>
+      <c r="G10" t="n">
         <v>4.7</v>
       </c>
-      <c r="F10" t="n">
+      <c r="H10" t="n">
         <v>23462.518</v>
       </c>
-      <c r="G10" t="n">
+      <c r="I10" t="n">
         <v>20219.111</v>
       </c>
-      <c r="H10" t="n">
+      <c r="J10" t="n">
         <v>16</v>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -1140,33 +1206,39 @@
         <v>117.9</v>
       </c>
       <c r="E11" t="n">
+        <v>56</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
         <v>3.4</v>
       </c>
-      <c r="F11" t="n">
+      <c r="H11" t="n">
         <v>11302.748</v>
       </c>
-      <c r="G11" t="n">
+      <c r="I11" t="n">
         <v>10183.353</v>
       </c>
-      <c r="H11" t="n">
+      <c r="J11" t="n">
         <v>11</v>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -1188,33 +1260,39 @@
         <v>69.8</v>
       </c>
       <c r="E12" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="F12" t="n">
+        <v>9</v>
+      </c>
+      <c r="G12" t="n">
         <v>2.6</v>
       </c>
-      <c r="F12" t="n">
+      <c r="H12" t="n">
         <v>1432.82</v>
       </c>
-      <c r="G12" t="n">
+      <c r="I12" t="n">
         <v>1422.999</v>
       </c>
-      <c r="H12" t="n">
+      <c r="J12" t="n">
         <v>0.7</v>
       </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -1236,33 +1314,39 @@
         <v>153.2</v>
       </c>
       <c r="E13" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="F13" t="n">
+        <v>5</v>
+      </c>
+      <c r="G13" t="n">
         <v>3.7</v>
       </c>
-      <c r="F13" t="n">
+      <c r="H13" t="n">
         <v>2029.733</v>
       </c>
-      <c r="G13" t="n">
+      <c r="I13" t="n">
         <v>1652.495</v>
       </c>
-      <c r="H13" t="n">
+      <c r="J13" t="n">
         <v>22.8</v>
       </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -1284,33 +1368,39 @@
         <v>73.2</v>
       </c>
       <c r="E14" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="F14" t="n">
+        <v>3</v>
+      </c>
+      <c r="G14" t="n">
         <v>5.1</v>
       </c>
-      <c r="F14" t="n">
+      <c r="H14" t="n">
         <v>12719.141</v>
       </c>
-      <c r="G14" t="n">
+      <c r="I14" t="n">
         <v>12859.585</v>
       </c>
-      <c r="H14" t="n">
+      <c r="J14" t="n">
         <v>-1.1</v>
       </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -1332,33 +1422,39 @@
         <v>104.1</v>
       </c>
       <c r="E15" t="n">
+        <v>52.7</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" t="n">
         <v>3.3</v>
       </c>
-      <c r="F15" t="n">
+      <c r="H15" t="n">
         <v>6973.333</v>
       </c>
-      <c r="G15" t="n">
+      <c r="I15" t="n">
         <v>6611.442</v>
       </c>
-      <c r="H15" t="n">
+      <c r="J15" t="n">
         <v>5.5</v>
       </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -1380,33 +1476,39 @@
         <v>69.8</v>
       </c>
       <c r="E16" t="n">
+        <v>42</v>
+      </c>
+      <c r="F16" t="n">
+        <v>2</v>
+      </c>
+      <c r="G16" t="n">
         <v>3.2</v>
       </c>
-      <c r="F16" t="n">
+      <c r="H16" t="n">
         <v>3238.387</v>
       </c>
-      <c r="G16" t="n">
+      <c r="I16" t="n">
         <v>3122.541</v>
       </c>
-      <c r="H16" t="n">
+      <c r="J16" t="n">
         <v>3.7</v>
       </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -1428,33 +1530,39 @@
         <v>91.5</v>
       </c>
       <c r="E17" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="F17" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" t="n">
         <v>3.8</v>
       </c>
-      <c r="F17" t="n">
+      <c r="H17" t="n">
         <v>2977.22</v>
       </c>
-      <c r="G17" t="n">
+      <c r="I17" t="n">
         <v>2910.717</v>
       </c>
-      <c r="H17" t="n">
+      <c r="J17" t="n">
         <v>2.3</v>
       </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -1476,33 +1584,39 @@
         <v>92</v>
       </c>
       <c r="E18" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
         <v>4.7</v>
       </c>
-      <c r="F18" t="n">
+      <c r="H18" t="n">
         <v>4606.864</v>
       </c>
-      <c r="G18" t="n">
+      <c r="I18" t="n">
         <v>4429.126</v>
       </c>
-      <c r="H18" t="n">
+      <c r="J18" t="n">
         <v>4</v>
       </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -1524,33 +1638,39 @@
         <v>42.1</v>
       </c>
       <c r="E19" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="F19" t="n">
+        <v>8</v>
+      </c>
+      <c r="G19" t="n">
         <v>4.4</v>
       </c>
-      <c r="F19" t="n">
+      <c r="H19" t="n">
         <v>4618.189</v>
       </c>
-      <c r="G19" t="n">
+      <c r="I19" t="n">
         <v>4666.998</v>
       </c>
-      <c r="H19" t="n">
+      <c r="J19" t="n">
         <v>-1</v>
       </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -1572,33 +1692,39 @@
         <v>123.1</v>
       </c>
       <c r="E20" t="n">
+        <v>64.90000000000001</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" t="n">
         <v>3.1</v>
       </c>
-      <c r="F20" t="n">
+      <c r="H20" t="n">
         <v>1414.874</v>
       </c>
-      <c r="G20" t="n">
+      <c r="I20" t="n">
         <v>1329.098</v>
       </c>
-      <c r="H20" t="n">
+      <c r="J20" t="n">
         <v>6.5</v>
       </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -1620,33 +1746,39 @@
         <v>65</v>
       </c>
       <c r="E21" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="F21" t="n">
+        <v>4</v>
+      </c>
+      <c r="G21" t="n">
         <v>4.3</v>
       </c>
-      <c r="F21" t="n">
+      <c r="H21" t="n">
         <v>6265.347</v>
       </c>
-      <c r="G21" t="n">
+      <c r="I21" t="n">
         <v>5988.528</v>
       </c>
-      <c r="H21" t="n">
+      <c r="J21" t="n">
         <v>4.6</v>
       </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -1668,33 +1800,39 @@
         <v>92.5</v>
       </c>
       <c r="E22" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" t="n">
         <v>4.4</v>
       </c>
-      <c r="F22" t="n">
+      <c r="H22" t="n">
         <v>7154.084</v>
       </c>
-      <c r="G22" t="n">
+      <c r="I22" t="n">
         <v>6797.484</v>
       </c>
-      <c r="H22" t="n">
+      <c r="J22" t="n">
         <v>5.2</v>
       </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -1716,33 +1854,39 @@
         <v>104</v>
       </c>
       <c r="E23" t="n">
+        <v>50.8</v>
+      </c>
+      <c r="F23" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" t="n">
         <v>5</v>
       </c>
-      <c r="F23" t="n">
+      <c r="H23" t="n">
         <v>10127.884</v>
       </c>
-      <c r="G23" t="n">
+      <c r="I23" t="n">
         <v>9934.483</v>
       </c>
-      <c r="H23" t="n">
+      <c r="J23" t="n">
         <v>1.9</v>
       </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -1764,33 +1908,39 @@
         <v>77.40000000000001</v>
       </c>
       <c r="E24" t="n">
+        <v>36.1</v>
+      </c>
+      <c r="F24" t="n">
+        <v>5</v>
+      </c>
+      <c r="G24" t="n">
         <v>4.4</v>
       </c>
-      <c r="F24" t="n">
+      <c r="H24" t="n">
         <v>5830.405</v>
       </c>
-      <c r="G24" t="n">
+      <c r="I24" t="n">
         <v>5484.002</v>
       </c>
-      <c r="H24" t="n">
+      <c r="J24" t="n">
         <v>6.3</v>
       </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -1812,33 +1962,39 @@
         <v>68.59999999999999</v>
       </c>
       <c r="E25" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="F25" t="n">
+        <v>4</v>
+      </c>
+      <c r="G25" t="n">
         <v>3.8</v>
       </c>
-      <c r="F25" t="n">
+      <c r="H25" t="n">
         <v>2954.16</v>
       </c>
-      <c r="G25" t="n">
+      <c r="I25" t="n">
         <v>2990.231</v>
       </c>
-      <c r="H25" t="n">
+      <c r="J25" t="n">
         <v>-1.2</v>
       </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -1860,33 +2016,39 @@
         <v>95.59999999999999</v>
       </c>
       <c r="E26" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" t="n">
         <v>3.7</v>
       </c>
-      <c r="F26" t="n">
+      <c r="H26" t="n">
         <v>6270.541</v>
       </c>
-      <c r="G26" t="n">
+      <c r="I26" t="n">
         <v>6075.411</v>
       </c>
-      <c r="H26" t="n">
+      <c r="J26" t="n">
         <v>3.2</v>
       </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -1908,33 +2070,39 @@
         <v>113.2</v>
       </c>
       <c r="E27" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="F27" t="n">
+        <v>3</v>
+      </c>
+      <c r="G27" t="n">
         <v>3.3</v>
       </c>
-      <c r="F27" t="n">
+      <c r="H27" t="n">
         <v>1144.694</v>
       </c>
-      <c r="G27" t="n">
+      <c r="I27" t="n">
         <v>1031.495</v>
       </c>
-      <c r="H27" t="n">
+      <c r="J27" t="n">
         <v>11</v>
       </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -1956,33 +2124,39 @@
         <v>93.2</v>
       </c>
       <c r="E28" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="F28" t="n">
+        <v>2</v>
+      </c>
+      <c r="G28" t="n">
         <v>2.9</v>
       </c>
-      <c r="F28" t="n">
+      <c r="H28" t="n">
         <v>2018.006</v>
       </c>
-      <c r="G28" t="n">
+      <c r="I28" t="n">
         <v>1892.059</v>
       </c>
-      <c r="H28" t="n">
+      <c r="J28" t="n">
         <v>6.7</v>
       </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -2004,33 +2178,39 @@
         <v>116.6</v>
       </c>
       <c r="E29" t="n">
+        <v>42.4</v>
+      </c>
+      <c r="F29" t="n">
+        <v>5</v>
+      </c>
+      <c r="G29" t="n">
         <v>5.1</v>
       </c>
-      <c r="F29" t="n">
+      <c r="H29" t="n">
         <v>3282.188</v>
       </c>
-      <c r="G29" t="n">
+      <c r="I29" t="n">
         <v>2868.531</v>
       </c>
-      <c r="H29" t="n">
+      <c r="J29" t="n">
         <v>14.4</v>
       </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -2052,33 +2232,39 @@
         <v>119.9</v>
       </c>
       <c r="E30" t="n">
+        <v>61.6</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" t="n">
         <v>2.9</v>
       </c>
-      <c r="F30" t="n">
+      <c r="H30" t="n">
         <v>1415.342</v>
       </c>
-      <c r="G30" t="n">
+      <c r="I30" t="n">
         <v>1337.48</v>
       </c>
-      <c r="H30" t="n">
+      <c r="J30" t="n">
         <v>5.8</v>
       </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -2100,33 +2286,39 @@
         <v>97.3</v>
       </c>
       <c r="E31" t="n">
+        <v>62.3</v>
+      </c>
+      <c r="F31" t="n">
+        <v>2</v>
+      </c>
+      <c r="G31" t="n">
         <v>4.5</v>
       </c>
-      <c r="F31" t="n">
+      <c r="H31" t="n">
         <v>9548.215</v>
       </c>
-      <c r="G31" t="n">
+      <c r="I31" t="n">
         <v>8870.312</v>
       </c>
-      <c r="H31" t="n">
+      <c r="J31" t="n">
         <v>7.6</v>
       </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -2148,33 +2340,39 @@
         <v>88.40000000000001</v>
       </c>
       <c r="E32" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="F32" t="n">
+        <v>3</v>
+      </c>
+      <c r="G32" t="n">
         <v>4.8</v>
       </c>
-      <c r="F32" t="n">
+      <c r="H32" t="n">
         <v>2125.498</v>
       </c>
-      <c r="G32" t="n">
+      <c r="I32" t="n">
         <v>2090.071</v>
       </c>
-      <c r="H32" t="n">
+      <c r="J32" t="n">
         <v>1.7</v>
       </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -2196,33 +2394,39 @@
         <v>95</v>
       </c>
       <c r="E33" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" t="n">
         <v>4.6</v>
       </c>
-      <c r="F33" t="n">
+      <c r="H33" t="n">
         <v>20002.427</v>
       </c>
-      <c r="G33" t="n">
+      <c r="I33" t="n">
         <v>19657.321</v>
       </c>
-      <c r="H33" t="n">
+      <c r="J33" t="n">
         <v>1.8</v>
       </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -2244,33 +2448,39 @@
         <v>114.9</v>
       </c>
       <c r="E34" t="n">
+        <v>59.3</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" t="n">
         <v>3.6</v>
       </c>
-      <c r="F34" t="n">
+      <c r="H34" t="n">
         <v>11197.968</v>
       </c>
-      <c r="G34" t="n">
+      <c r="I34" t="n">
         <v>10037.218</v>
       </c>
-      <c r="H34" t="n">
+      <c r="J34" t="n">
         <v>11.6</v>
       </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -2292,33 +2502,39 @@
         <v>49.2</v>
       </c>
       <c r="E35" t="n">
+        <v>35</v>
+      </c>
+      <c r="F35" t="n">
+        <v>9</v>
+      </c>
+      <c r="G35" t="n">
         <v>2.3</v>
       </c>
-      <c r="F35" t="n">
+      <c r="H35" t="n">
         <v>799.3579999999999</v>
       </c>
-      <c r="G35" t="n">
+      <c r="I35" t="n">
         <v>755.537</v>
       </c>
-      <c r="H35" t="n">
+      <c r="J35" t="n">
         <v>5.8</v>
       </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -2340,33 +2556,39 @@
         <v>102.9</v>
       </c>
       <c r="E36" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="F36" t="n">
+        <v>2</v>
+      </c>
+      <c r="G36" t="n">
         <v>3.6</v>
       </c>
-      <c r="F36" t="n">
+      <c r="H36" t="n">
         <v>11900.51</v>
       </c>
-      <c r="G36" t="n">
+      <c r="I36" t="n">
         <v>11622.315</v>
       </c>
-      <c r="H36" t="n">
+      <c r="J36" t="n">
         <v>2.4</v>
       </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -2388,33 +2610,39 @@
         <v>76.5</v>
       </c>
       <c r="E37" t="n">
+        <v>44.6</v>
+      </c>
+      <c r="F37" t="n">
+        <v>3</v>
+      </c>
+      <c r="G37" t="n">
         <v>4.2</v>
       </c>
-      <c r="F37" t="n">
+      <c r="H37" t="n">
         <v>4123.288</v>
       </c>
-      <c r="G37" t="n">
+      <c r="I37" t="n">
         <v>3910.518</v>
       </c>
-      <c r="H37" t="n">
+      <c r="J37" t="n">
         <v>5.4</v>
       </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -2436,33 +2664,39 @@
         <v>85.09999999999999</v>
       </c>
       <c r="E38" t="n">
+        <v>31</v>
+      </c>
+      <c r="F38" t="n">
+        <v>5</v>
+      </c>
+      <c r="G38" t="n">
         <v>5.2</v>
       </c>
-      <c r="F38" t="n">
+      <c r="H38" t="n">
         <v>4273.586</v>
       </c>
-      <c r="G38" t="n">
+      <c r="I38" t="n">
         <v>4018.542</v>
       </c>
-      <c r="H38" t="n">
+      <c r="J38" t="n">
         <v>6.3</v>
       </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -2484,33 +2718,39 @@
         <v>86.90000000000001</v>
       </c>
       <c r="E39" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="F39" t="n">
+        <v>2</v>
+      </c>
+      <c r="G39" t="n">
         <v>4.1</v>
       </c>
-      <c r="F39" t="n">
+      <c r="H39" t="n">
         <v>13059.432</v>
       </c>
-      <c r="G39" t="n">
+      <c r="I39" t="n">
         <v>12789.838</v>
       </c>
-      <c r="H39" t="n">
+      <c r="J39" t="n">
         <v>2.1</v>
       </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -2532,33 +2772,39 @@
         <v>119.3</v>
       </c>
       <c r="E40" t="n">
+        <v>61.3</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" t="n">
         <v>4.1</v>
       </c>
-      <c r="F40" t="n">
+      <c r="H40" t="n">
         <v>1114.521</v>
       </c>
-      <c r="G40" t="n">
+      <c r="I40" t="n">
         <v>1056.886</v>
       </c>
-      <c r="H40" t="n">
+      <c r="J40" t="n">
         <v>5.5</v>
       </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -2580,33 +2826,39 @@
         <v>115.2</v>
       </c>
       <c r="E41" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" t="n">
         <v>4.4</v>
       </c>
-      <c r="F41" t="n">
+      <c r="H41" t="n">
         <v>5570.274</v>
       </c>
-      <c r="G41" t="n">
+      <c r="I41" t="n">
         <v>4896.006</v>
       </c>
-      <c r="H41" t="n">
+      <c r="J41" t="n">
         <v>13.8</v>
       </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -2628,33 +2880,39 @@
         <v>91.8</v>
       </c>
       <c r="E42" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="F42" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" t="n">
         <v>2</v>
       </c>
-      <c r="F42" t="n">
+      <c r="H42" t="n">
         <v>935.0940000000001</v>
       </c>
-      <c r="G42" t="n">
+      <c r="I42" t="n">
         <v>854.663</v>
       </c>
-      <c r="H42" t="n">
+      <c r="J42" t="n">
         <v>9.4</v>
       </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -2676,33 +2934,39 @@
         <v>122.5</v>
       </c>
       <c r="E43" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="F43" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" t="n">
         <v>3.5</v>
       </c>
-      <c r="F43" t="n">
+      <c r="H43" t="n">
         <v>7315.076</v>
       </c>
-      <c r="G43" t="n">
+      <c r="I43" t="n">
         <v>6595.354</v>
       </c>
-      <c r="H43" t="n">
+      <c r="J43" t="n">
         <v>10.9</v>
       </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -2724,33 +2988,39 @@
         <v>91.2</v>
       </c>
       <c r="E44" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="F44" t="n">
+        <v>2</v>
+      </c>
+      <c r="G44" t="n">
         <v>4.4</v>
       </c>
-      <c r="F44" t="n">
+      <c r="H44" t="n">
         <v>31709.821</v>
       </c>
-      <c r="G44" t="n">
+      <c r="I44" t="n">
         <v>27468.531</v>
       </c>
-      <c r="H44" t="n">
+      <c r="J44" t="n">
         <v>15.4</v>
       </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -2772,33 +3042,39 @@
         <v>124.3</v>
       </c>
       <c r="E45" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="F45" t="n">
+        <v>4</v>
+      </c>
+      <c r="G45" t="n">
         <v>3.6</v>
       </c>
-      <c r="F45" t="n">
+      <c r="H45" t="n">
         <v>3538.904</v>
       </c>
-      <c r="G45" t="n">
+      <c r="I45" t="n">
         <v>2983.626</v>
       </c>
-      <c r="H45" t="n">
+      <c r="J45" t="n">
         <v>18.6</v>
       </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -2820,33 +3096,39 @@
         <v>99.5</v>
       </c>
       <c r="E46" t="n">
+        <v>61.7</v>
+      </c>
+      <c r="F46" t="n">
+        <v>4</v>
+      </c>
+      <c r="G46" t="n">
         <v>2.6</v>
       </c>
-      <c r="F46" t="n">
+      <c r="H46" t="n">
         <v>644.663</v>
       </c>
-      <c r="G46" t="n">
+      <c r="I46" t="n">
         <v>625.8099999999999</v>
       </c>
-      <c r="H46" t="n">
+      <c r="J46" t="n">
         <v>3</v>
       </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -2868,33 +3150,39 @@
         <v>83.3</v>
       </c>
       <c r="E47" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="F47" t="n">
+        <v>2</v>
+      </c>
+      <c r="G47" t="n">
         <v>3.7</v>
       </c>
-      <c r="F47" t="n">
+      <c r="H47" t="n">
         <v>8880.107</v>
       </c>
-      <c r="G47" t="n">
+      <c r="I47" t="n">
         <v>8367.303</v>
       </c>
-      <c r="H47" t="n">
+      <c r="J47" t="n">
         <v>6.1</v>
       </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -2916,33 +3204,39 @@
         <v>111.8</v>
       </c>
       <c r="E48" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="F48" t="n">
+        <v>5</v>
+      </c>
+      <c r="G48" t="n">
         <v>5.2</v>
       </c>
-      <c r="F48" t="n">
+      <c r="H48" t="n">
         <v>8001.02</v>
       </c>
-      <c r="G48" t="n">
+      <c r="I48" t="n">
         <v>7167.287</v>
       </c>
-      <c r="H48" t="n">
+      <c r="J48" t="n">
         <v>11.6</v>
       </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -2964,33 +3258,39 @@
         <v>64.7</v>
       </c>
       <c r="E49" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="F49" t="n">
+        <v>7</v>
+      </c>
+      <c r="G49" t="n">
         <v>4.2</v>
       </c>
-      <c r="F49" t="n">
+      <c r="H49" t="n">
         <v>1766.147</v>
       </c>
-      <c r="G49" t="n">
+      <c r="I49" t="n">
         <v>1843.332</v>
       </c>
-      <c r="H49" t="n">
+      <c r="J49" t="n">
         <v>-4.2</v>
       </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -3012,33 +3312,39 @@
         <v>102.5</v>
       </c>
       <c r="E50" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="F50" t="n">
+        <v>1</v>
+      </c>
+      <c r="G50" t="n">
         <v>3.3</v>
       </c>
-      <c r="F50" t="n">
+      <c r="H50" t="n">
         <v>5972.787</v>
       </c>
-      <c r="G50" t="n">
+      <c r="I50" t="n">
         <v>5762.927</v>
       </c>
-      <c r="H50" t="n">
+      <c r="J50" t="n">
         <v>3.6</v>
       </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>
@@ -3060,33 +3366,39 @@
         <v>75.09999999999999</v>
       </c>
       <c r="E51" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="F51" t="n">
+        <v>7</v>
+      </c>
+      <c r="G51" t="n">
         <v>3.2</v>
       </c>
-      <c r="F51" t="n">
+      <c r="H51" t="n">
         <v>588.753</v>
       </c>
-      <c r="G51" t="n">
+      <c r="I51" t="n">
         <v>586.389</v>
       </c>
-      <c r="H51" t="n">
+      <c r="J51" t="n">
         <v>0.4</v>
       </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>2016-01-01</t>
-        </is>
-      </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
         <is>
           <t>2025-01-01</t>
         </is>

</xml_diff>